<commit_message>
refactor: replace forbidden list with blocked_name table
- Remove forbidden list from login server config
- Add blocked_name table support in model
- Rename 'allow other language' to 'allow_foreign_name'
- Update config defaults (admin_mode to false)
- Reorder GENDER enum in model generation
- Update model generation timestamp
</commit_message>
<xml_diff>
--- a/resources/table/preset.xlsx
+++ b/resources/table/preset.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\fb\resources\table\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\fb\resources\table\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA613AC0-3F3E-4998-98E1-E1F802A4D955}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA835BFC-4D98-4F0E-AC43-A173A2352D63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{2AD1A0EA-2C47-4BED-8190-24EDA4F164BF}"/>
+    <workbookView xWindow="38280" yWindow="-135" windowWidth="38640" windowHeight="21120" xr2:uid="{2AD1A0EA-2C47-4BED-8190-24EDA4F164BF}"/>
   </bookViews>
   <sheets>
     <sheet name="preset" sheetId="7" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="25">
   <si>
     <t>id</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -120,6 +120,10 @@
   </si>
   <si>
     <t>GENDER</t>
+  </si>
+  <si>
+    <t>gender</t>
+    <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -182,7 +186,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="표준" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -198,7 +202,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 테마">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
     <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
@@ -507,7 +511,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>14</v>

</xml_diff>